<commit_message>
Adding 200+ labeled videos
</commit_message>
<xml_diff>
--- a/Data/Transplants_Team_Master_File.xlsx
+++ b/Data/Transplants_Team_Master_File.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/99ca9685b2417778/Documentos/CMU - Heinz College/Coursework/Semester III/Capstone Project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/99ca9685b2417778/Documentos/CMU - Heinz College/Coursework/Semester III/Capstone Project/Repo/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="1" documentId="11_35F5C9A31049260E62355476585DCE3A8745DFD1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2300F1C5-BB53-4FEF-86E3-49E9A593D4C8}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="21840" yWindow="-4809" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3573,6 +3573,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>